<commit_message>
Refresh the fabrication exports
Regenerated output job data, mostly for the Digital LED load board
(Gerbers, BOM and the JLC BOM/CPL pair). The Controller and RGBW Gerber
archives only differ in their zip timestamps.
</commit_message>
<xml_diff>
--- a/Hardware/DALI_Load_250W_DigitalLED/JLC_PCBA_BOM-DALI_LOAD_DigitalLED(V0.1).xlsx
+++ b/Hardware/DALI_Load_250W_DigitalLED/JLC_PCBA_BOM-DALI_LOAD_DigitalLED(V0.1).xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="111">
   <si>
     <t xml:space="preserve">Comment</t>
   </si>
@@ -157,6 +157,19 @@
     <t xml:space="preserve">SOT95P280X110-6N (SOT23-6L)</t>
   </si>
   <si>
+    <t xml:space="preserve">FFC 0.5mm 10Pin 90°</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FFC 0.5mm 10P Bottom Connection
+C262659</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TE_1-1734592-0</t>
+  </si>
+  <si>
     <t xml:space="preserve">NLCV32T-100K-PF (10uH)</t>
   </si>
   <si>
@@ -304,6 +317,9 @@
     <t xml:space="preserve">C5123971</t>
   </si>
   <si>
+    <t xml:space="preserve">C262659</t>
+  </si>
+  <si>
     <t xml:space="preserve">C107341</t>
   </si>
   <si>
@@ -323,6 +339,21 @@
   </si>
   <si>
     <t xml:space="preserve">C25741</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C23196</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C22809</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C22966</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C22808</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C970946</t>
   </si>
 </sst>
 </file>
@@ -615,7 +646,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <sheetPr/>
-  <dimension ref="A1:F27"/>
+  <dimension ref="A1:F28"/>
   <sheetFormatPr defaultRowHeight="12.75"/>
   <cols>
     <col min="1" max="5" width="20.2109375" customWidth="1"/>
@@ -638,7 +669,7 @@
         <v>5</v>
       </c>
       <c r="F1" s="34" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -692,7 +723,7 @@
         <v>3</v>
       </c>
       <c r="F4" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -712,7 +743,7 @@
         <v>2</v>
       </c>
       <c r="F5" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -732,7 +763,7 @@
         <v>2</v>
       </c>
       <c r="F6" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
     </row>
     <row r="7" spans="1:5">
@@ -752,7 +783,7 @@
         <v>1</v>
       </c>
       <c r="F7" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
     </row>
     <row r="8" spans="1:5">
@@ -789,7 +820,7 @@
         <v>3</v>
       </c>
       <c r="F9" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
     </row>
     <row r="10" spans="1:5">
@@ -826,7 +857,7 @@
         <v>1</v>
       </c>
       <c r="F11" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
     </row>
     <row r="12" spans="1:5">
@@ -846,7 +877,7 @@
         <v>1</v>
       </c>
       <c r="F12" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
     </row>
     <row r="13" spans="1:5">
@@ -866,7 +897,7 @@
         <v>1</v>
       </c>
       <c r="F13" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
     </row>
     <row r="14" spans="1:5">
@@ -874,30 +905,33 @@
         <v>49</v>
       </c>
       <c r="B14" s="19" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C14" s="17" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D14" s="17" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E14" s="32">
         <v>1</v>
+      </c>
+      <c r="F14" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="15" spans="1:5">
       <c r="A15" s="31" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B15" s="19" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C15" s="17" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D15" s="17" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E15" s="32">
         <v>1</v>
@@ -905,16 +939,16 @@
     </row>
     <row r="16" spans="1:5">
       <c r="A16" s="31" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B16" s="19" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C16" s="17" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D16" s="17" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E16" s="32">
         <v>1</v>
@@ -922,7 +956,7 @@
     </row>
     <row r="17" spans="1:5">
       <c r="A17" s="31" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B17" s="19" t="s">
         <v>59</v>
@@ -935,9 +969,6 @@
       </c>
       <c r="E17" s="32">
         <v>1</v>
-      </c>
-      <c r="F17" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="18" spans="1:5">
@@ -956,173 +987,208 @@
       <c r="E18" s="32">
         <v>1</v>
       </c>
+      <c r="F18" t="s">
+        <v>100</v>
+      </c>
     </row>
     <row r="19" spans="1:5">
       <c r="A19" s="31" t="s">
         <v>66</v>
       </c>
       <c r="B19" s="19" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="C19" s="17" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D19" s="17" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="E19" s="32">
         <v>1</v>
+      </c>
+      <c r="F19" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="20" spans="1:5">
       <c r="A20" s="31" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B20" s="19" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="C20" s="17" t="s">
+        <v>71</v>
+      </c>
+      <c r="D20" s="17" t="s">
         <v>69</v>
       </c>
-      <c r="D20" s="17" t="s">
-        <v>70</v>
-      </c>
       <c r="E20" s="32">
         <v>1</v>
       </c>
       <c r="F20" t="s">
-        <v>96</v>
+        <v>107</v>
       </c>
     </row>
     <row r="21" spans="1:5">
       <c r="A21" s="31" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B21" s="19" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="C21" s="17" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D21" s="17" t="s">
-        <v>65</v>
+        <v>74</v>
       </c>
       <c r="E21" s="32">
         <v>1</v>
+      </c>
+      <c r="F21" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="22" spans="1:5">
       <c r="A22" s="31" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B22" s="19" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="C22" s="17" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D22" s="17" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="E22" s="32">
         <v>1</v>
+      </c>
+      <c r="F22" t="s">
+        <v>108</v>
       </c>
     </row>
     <row r="23" spans="1:5">
       <c r="A23" s="31" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B23" s="19" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="C23" s="17" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D23" s="17" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="E23" s="32">
         <v>1</v>
       </c>
       <c r="F23" t="s">
-        <v>97</v>
+        <v>109</v>
       </c>
     </row>
     <row r="24" spans="1:5">
       <c r="A24" s="31" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B24" s="19" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="C24" s="17" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="D24" s="17" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="E24" s="32">
         <v>1</v>
       </c>
       <c r="F24" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
     </row>
     <row r="25" spans="1:5">
       <c r="A25" s="31" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B25" s="19" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="C25" s="17" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="D25" s="17" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E25" s="32">
         <v>1</v>
       </c>
       <c r="F25" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
     </row>
     <row r="26" spans="1:5">
       <c r="A26" s="31" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B26" s="19" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="C26" s="17" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D26" s="17" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="E26" s="32">
         <v>1</v>
       </c>
       <c r="F26" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
     </row>
     <row r="27" spans="1:5">
       <c r="A27" s="31" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B27" s="19" t="s">
-        <v>84</v>
+        <v>67</v>
       </c>
       <c r="C27" s="17" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D27" s="17" t="s">
-        <v>86</v>
+        <v>74</v>
       </c>
       <c r="E27" s="32">
         <v>1</v>
+      </c>
+      <c r="F27" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5">
+      <c r="A28" s="31" t="s">
+        <v>87</v>
+      </c>
+      <c r="B28" s="19" t="s">
+        <v>88</v>
+      </c>
+      <c r="C28" s="17" t="s">
+        <v>89</v>
+      </c>
+      <c r="D28" s="17" t="s">
+        <v>90</v>
+      </c>
+      <c r="E28" s="32">
+        <v>1</v>
+      </c>
+      <c r="F28" t="s">
+        <v>110</v>
       </c>
     </row>
   </sheetData>

</xml_diff>